<commit_message>
Merged PR 2519: Merge planningmodulenewscenarios to master
Added New test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Organizational_SiteVisit_Field_Values.xlsx
+++ b/src/main/resources/Organizational_SiteVisit_Field_Values.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nauman.shahid/Nauman-data/Dev_Home/govgrants-product-automation/src/main/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F675D27-1538-E347-876D-800BBE2B70D7}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49227B2D-EFAF-45AA-AB3E-6D604244D98D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4000" yWindow="-17560" windowWidth="23260" windowHeight="12580" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="7" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId2"/>
-    <sheet name="Edition" sheetId="3" r:id="rId3"/>
-    <sheet name="Form Fields" sheetId="5" r:id="rId4"/>
+    <sheet name="Fiscal" sheetId="6" r:id="rId3"/>
+    <sheet name="Edition" sheetId="3" r:id="rId4"/>
+    <sheet name="Form Fields" sheetId="5" r:id="rId5"/>
+    <sheet name="Program" sheetId="7" r:id="rId6"/>
+    <sheet name="Application" sheetId="8" r:id="rId7"/>
+    <sheet name="Award" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -28,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="52">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -168,13 +172,22 @@
     <t xml:space="preserve"> hiring is to occur, does the agency adhere to Federal and State EEOC (Equal employment Opportunity Act) policies and procedures</t>
   </si>
   <si>
-    <t>Automation Site Visit</t>
-  </si>
-  <si>
     <t>SiteVisitType__c</t>
   </si>
   <si>
     <t>Award</t>
+  </si>
+  <si>
+    <t>Fiscal</t>
+  </si>
+  <si>
+    <t>Automation Site Visit Org level</t>
+  </si>
+  <si>
+    <t>Program</t>
+  </si>
+  <si>
+    <t>Application</t>
   </si>
 </sst>
 </file>
@@ -534,13 +547,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -551,7 +564,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -559,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -573,7 +586,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -584,15 +597,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="s">
         <v>47</v>
-      </c>
-      <c r="C5" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -603,12 +616,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -616,7 +629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -624,7 +637,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -632,7 +645,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -640,22 +653,22 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>27</v>
       </c>
@@ -666,16 +679,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A2DDC02-74D6-4569-851C-F07FFE02569B}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" style="1"/>
+    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -686,81 +700,48 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -769,16 +750,119 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F8298A-0165-44BF-9061-10BEE0A93A27}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.33203125" customWidth="1"/>
-    <col min="3" max="3" width="100.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="100.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -789,7 +873,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -800,7 +884,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -811,7 +895,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -822,7 +906,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -833,7 +917,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -844,7 +928,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -855,7 +939,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -866,7 +950,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -877,7 +961,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -886,6 +970,219 @@
       </c>
       <c r="C10" t="s">
         <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A304E392-7396-448A-86B5-CCFD1BE04B95}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.77734375" style="1"/>
+    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02608AAB-67CB-461D-B36D-03C96B96BB37}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.77734375" style="1"/>
+    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33F18BA5-C512-4E65-B599-8A11292F0D8E}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.77734375" style="1"/>
+    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>